<commit_message>
Atualiza planilha: Render grátis, investimento único R$ 210 para lançamento em 01/06/2026
</commit_message>
<xml_diff>
--- a/custos_mensais_aquiresolve.xlsx
+++ b/custos_mensais_aquiresolve.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,6 +51,29 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00C00000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00375623"/>
       <sz val="10"/>
     </font>
@@ -82,14 +105,8 @@
       <color rgb="002F5496"/>
       <sz val="12"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00C00000"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -100,6 +117,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="002F5496"/>
         <bgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -127,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -145,21 +168,27 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -525,14 +554,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -593,18 +622,18 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Starter (US$ 7/mês)</t>
+          <t>Plano Gratuito (Free)</t>
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>456</v>
+        <v>0</v>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Plano básico pago. Web service sempre ativo (sem hibernação). 512MB RAM, 0.5 CPU, largura de banda inclusa.</t>
+          <t>Web service gratuito. Hiberna após 15 min de inatividade, mas suficiente para MVP no lançamento.</t>
         </is>
       </c>
     </row>
@@ -616,18 +645,18 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Basic-256mb (US$ 7/mês)</t>
+          <t>Plano Gratuito (Free - 90 dias)</t>
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>456</v>
+        <v>0</v>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Banco PostgreSQL gerenciado. 256MB RAM, 0.1 CPU, 1GB armazenamento. Suficiente para início.</t>
+          <t>PostgreSQL grátis por 90 dias. Após esse período, plano Basic-256mb (~R$ 38/mês).</t>
         </is>
       </c>
     </row>
@@ -639,7 +668,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>registro.br</t>
+          <t>registro.br (2 anos)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
@@ -650,68 +679,96 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>R$ 149,90 a cada 2 anos (não é mensal). Valor rateado em 24 meses para referência: R$ 149,90 ÷ 24 = R$ 6,25/mês.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+          <t>R$ 149,90 a cada 2 anos (pagamento único). Rateio: R$ 149,90 ÷ 24 = R$ 6,25/mês para referência mensal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="55" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>SUBTOTAL (recorrente mensal)</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="n"/>
+          <t>INVESTIMENTO INICIAL (lançamento)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Único - Maio/Junho 2026</t>
+        </is>
+      </c>
       <c r="C6" s="8" t="n">
-        <v>121</v>
-      </c>
-      <c r="D6" s="8" t="n">
-        <v>1452</v>
+        <v>210</v>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Único</t>
+        </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Firebase + Render (API + PostgreSQL)</t>
+          <t>Ferramentas de desenvolvimento necessárias para lançar o app até 01/06/2026. Inclui: assinaturas de ferramentas (ex: conta Google Play Developer R$ 120, hospedagem de assets, testes, etc.). Pagamento único.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>TOTAL GERAL (com domínio rateado)</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="8" t="n">
-        <v>127.25</v>
-      </c>
-      <c r="D7" s="8" t="n">
-        <v>1527</v>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>Domínio rateado em 24 meses (R$ 149,90 ÷ 24 = R$ 6,25/mês)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+          <t>TOTAL RECORRENTE (mensal)</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="12" t="n">
+        <v>51.25</v>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>615</v>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Firebase R$ 45 + Render grátis + Domínio rateado R$ 6,25</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="35" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>CUSTO PRIMEIRO MÊS (Junho/2026)</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n"/>
+      <c r="C8" s="8" t="n">
+        <v>261.25</v>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Mensal R$ 51,25 + Investimento único R$ 210,00 = R$ 261,25 no primeiro mês.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Notas:</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="110" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>• Firebase Blaze: faturamento via Google Cloud. Os primeiros 50K leituras/dia, 20K escritas/dia e 1GB armazenamento são gratuitos. R$ 45/mês é estimativa para app com ~1.000 usuários ativos.
-• Render Starter: US$ 7/mês por serviço (API = US$ 7 + PostgreSQL = US$ 7). Cotação US$ 1 ≈ R$ 5,40 (maio/2026).
-• Domínio: R$ 149,90 a cada 2 anos (pagamento único no registro.br). O valor de R$ 6,25/mês é apenas uma referência de rateio.
-• Estes valores são baseados nos planos públicos atuais (maio/2026) e podem variar conforme uso do app.</t>
+    <row r="11" ht="120" customHeight="1">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>• Firebase Blaze: faturamento via Google Cloud. 50K leituras/dia, 20K escritas/dia e 1GB armazenamento gratuitos. R$ 45/mês é estimativa para app com ~1.000 usuários ativos.
+• Render: plano gratuito por 90 dias para o PostgreSQL. Web service gratuito (hiberna após 15 min). Custo zero no lançamento.
+• Domínio: R$ 149,90 a cada 2 anos (pagamento único no registro.br). R$ 6,25/mês é apenas rateio ilustrativo.
+• Investimento único de R$ 210,00: ferramentas de desenvolvimento para lançar até 01/06/2026.
+• Cotação US$ 1 ≈ R$ 5,40 (maio/2026).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A11:E11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -723,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -731,77 +788,77 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Detalhamento - Domínio</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>Registro</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>registro.br</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Valor total (2 anos)</t>
         </is>
       </c>
-      <c r="B3" s="15" t="n">
+      <c r="B3" s="19" t="n">
         <v>149.9</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>Periodicidade</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>A cada 2 anos (pagamento único)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Valor mensal (referência)</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="20" t="n">
         <v>6.25</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Próximo vencimento</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Conforme data de registro</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>IMPORTANTE:</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="9" ht="75" customHeight="1">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>O domínio .com.br é pago no registro.br a cada 2 anos no valor de R$ 149,90. Não há cobrança mensal recorrente. O valor de R$ 6,25/mês exibido na planilha principal é apenas um rateio ilustrativo (R$ 149,90 ÷ 24 meses) para facilitar o planejamento financeiro mensal.</t>
         </is>
@@ -810,9 +867,10 @@
     <row r="10"/>
     <row r="11"/>
     <row r="12"/>
+    <row r="13"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A9:B12"/>
+    <mergeCell ref="A9:B13"/>
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>